<commit_message>
Add 01-1_Under_Hero sheet to all 5 category Excel files
Add the under-hero blocks sheet (Name/Text) missing vs the template sample,
positioned after 01_SECTION_UF, with content adapted per category
(Косметология, IPL-терапия, RF-лифтинг, Лазерные аппараты, Фототерапия).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012Rw9dvcAKokoAsKsBSt35U
</commit_message>
<xml_diff>
--- a/medford_fototerapiya_v1.xlsx
+++ b/medford_fototerapiya_v1.xlsx
@@ -9,16 +9,17 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_README" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_SECTION_UF" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_BLOCKS" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_PRODUCTS" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_COMPARE_ROWS" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_CONTENT_ITEMS" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_WAVELENGTHS" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_RATING" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_CASES" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_FAQ" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_FIELD_MAP" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_ENUMS" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01-1_Under_Hero" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_BLOCKS" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_PRODUCTS" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_COMPARE_ROWS" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_CONTENT_ITEMS" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_WAVELENGTHS" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_RATING" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_CASES" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_FAQ" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_FIELD_MAP" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_ENUMS" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -780,6 +781,193 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:N5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="30" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>08_CASES — Кейсы (ПЛЕЙСХОЛДЕРЫ, заполнить вручную)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>IBLOCK_ID</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>ELEMENT_XML_ID</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>ACTIVE *</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>SORT *</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>NAME *</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>PROPERTY_SECTION_CODE *</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>PROPERTY_BLOCK_CODE *</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>PROPERTY_CASE_PAGE_URL *</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTY_CARD_TITLE_OVERRIDE</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTY_LABEL_OVERRIDE</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTY_CLINIC_OVERRIDE</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTY_EQUIPMENT_OVERRIDE</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTY_DELIVERY_TIME_OVERRIDE</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTY_SERVICES_OVERRIDE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>CASE_PHOTO_1</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>[Кейс: LED-фототерапия в клинике]</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>fototerapiya</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>CASES</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>[URL кейса]</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>[Оснащение клиники — Decotica Curelux]</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>[Проект, год]</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>[Клиника, город]</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>[Decotica Curelux]</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>[срок]</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>Подбор, монтаж, обучение, сервис</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>ACTIVE=N: активировать после заполнения реальными данными.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1154,7 +1342,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2006,7 +2194,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3056,6 +3244,85 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="B1:C5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Ввод в эксплуатацию</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Проведём пусконаладку, настройку длин волн и SMART-протоколов, обучение работе</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Подготовка КП за 1 день</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Обратный звонок бесплатно</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Сервисное обслуживание и гарантия</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Гарантийное сопровождение и диагностика; LED-фототерапия работает без расходных материалов</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Подбор решения</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Подберём аппарат фототерапии под задачи клиники и программы восстановления</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3526,7 +3793,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3863,7 +4130,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4229,7 +4496,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5333,7 +5600,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5613,7 +5880,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5756,191 +6023,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:N5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="36" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="30" customWidth="1" min="14" max="14"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>08_CASES — Кейсы (ПЛЕЙСХОЛДЕРЫ, заполнить вручную)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>IBLOCK_ID</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>ELEMENT_XML_ID</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>ACTIVE *</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>SORT *</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>NAME *</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>PROPERTY_SECTION_CODE *</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>PROPERTY_BLOCK_CODE *</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>PROPERTY_CASE_PAGE_URL *</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>PROPERTY_CARD_TITLE_OVERRIDE</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>PROPERTY_LABEL_OVERRIDE</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>PROPERTY_CLINIC_OVERRIDE</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>PROPERTY_EQUIPMENT_OVERRIDE</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>PROPERTY_DELIVERY_TIME_OVERRIDE</t>
-        </is>
-      </c>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>PROPERTY_SERVICES_OVERRIDE</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="n">
-        <v>21</v>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>CASE_PHOTO_1</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>[Кейс: LED-фототерапия в клинике]</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>fototerapiya</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>CASES</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>[URL кейса]</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>[Оснащение клиники — Decotica Curelux]</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>[Проект, год]</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>[Клиника, город]</t>
-        </is>
-      </c>
-      <c r="L4" s="3" t="inlineStr">
-        <is>
-          <t>[Decotica Curelux]</t>
-        </is>
-      </c>
-      <c r="M4" s="3" t="inlineStr">
-        <is>
-          <t>[срок]</t>
-        </is>
-      </c>
-      <c r="N4" s="3" t="inlineStr">
-        <is>
-          <t>Подбор, монтаж, обучение, сервис</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>ACTIVE=N: активировать после заполнения реальными данными.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:N1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>